<commit_message>
consertando o levenberg, o testeo2copy da f1 ta funcionando
</commit_message>
<xml_diff>
--- a/fuction_ensemble_1/redes-ensemble-s/Teste02 copy/content/results/metrics_1_3.xlsx
+++ b/fuction_ensemble_1/redes-ensemble-s/Teste02 copy/content/results/metrics_1_3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q26"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,1376 +513,1046 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_10</t>
+          <t>model_1_3_13</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8073783302276021</v>
+        <v>0.3665618702355821</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3960099834619338</v>
+        <v>-0.0966691057973228</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7570856816465078</v>
+        <v>-3.413522500801603</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4786571646126593</v>
+        <v>-0.465139394851684</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6808445152478331</v>
+        <v>-0.36117486688401</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1143485439997712</v>
+        <v>0.3760362369305901</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3585545648271732</v>
+        <v>0.6510301548399551</v>
       </c>
       <c r="I2" t="n">
-        <v>0.1184153695257059</v>
+        <v>0.3888497136915866</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2521184770068</v>
+        <v>0.6717707074809345</v>
       </c>
       <c r="K2" t="n">
-        <v>0.185266923266253</v>
+        <v>0.5303102105862605</v>
       </c>
       <c r="L2" t="n">
-        <v>0.1758701047744956</v>
+        <v>0.3667508332474741</v>
       </c>
       <c r="M2" t="n">
-        <v>0.3381546155233892</v>
+        <v>0.6132179359172317</v>
       </c>
       <c r="N2" t="n">
-        <v>0.4863422139402722</v>
+        <v>-0.6891683460384477</v>
       </c>
       <c r="O2" t="n">
-        <v>0.3525505575827745</v>
+        <v>0.639323892985352</v>
       </c>
       <c r="P2" t="n">
-        <v>34.33700818286838</v>
+        <v>31.9561395308412</v>
       </c>
       <c r="Q2" t="n">
-        <v>52.62014555589139</v>
+        <v>50.2392769038642</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_12</t>
+          <t>model_1_3_14</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8072748738529221</v>
+        <v>0.3860893063222024</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3907486651107778</v>
+        <v>-0.106787715346935</v>
       </c>
       <c r="D3" t="n">
-        <v>0.7457479988188753</v>
+        <v>-4.305149523393086</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4645408776870319</v>
+        <v>-0.2347821837590287</v>
       </c>
       <c r="F3" t="n">
-        <v>0.670204018610303</v>
+        <v>-0.3264423438514328</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1144099601728639</v>
+        <v>0.3644439073282559</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3616779106775381</v>
+        <v>0.6570369985697779</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1239422397023977</v>
+        <v>0.4674057678164742</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2589450343489297</v>
+        <v>0.5661512509208213</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1914436370256637</v>
+        <v>0.5167785093686478</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1803900782855624</v>
+        <v>0.3499791278111303</v>
       </c>
       <c r="M3" t="n">
-        <v>0.3382454141194879</v>
+        <v>0.6036918976831277</v>
       </c>
       <c r="N3" t="n">
-        <v>0.4860663302744589</v>
+        <v>-0.6370951831407936</v>
       </c>
       <c r="O3" t="n">
-        <v>0.3526452216630882</v>
+        <v>0.6293923115820045</v>
       </c>
       <c r="P3" t="n">
-        <v>34.33593427875643</v>
+        <v>32.01876525747134</v>
       </c>
       <c r="Q3" t="n">
-        <v>52.61907165177944</v>
+        <v>50.30190263049435</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_15</t>
+          <t>model_1_3_12</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.806394484149203</v>
+        <v>0.362548150317858</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3904148052163144</v>
+        <v>-0.1144388319291314</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7419461689759466</v>
+        <v>-3.344556165772955</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4502026206931821</v>
+        <v>-0.4914999744590838</v>
       </c>
       <c r="F4" t="n">
-        <v>0.6626352473202701</v>
+        <v>-0.3688881902202394</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1149325975318465</v>
+        <v>0.3784189544574237</v>
       </c>
       <c r="H4" t="n">
-        <v>0.361876104332888</v>
+        <v>0.6615790318839966</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1257955478514429</v>
+        <v>0.3827734923456261</v>
       </c>
       <c r="J4" t="n">
-        <v>0.2658789351735872</v>
+        <v>0.6838571105049028</v>
       </c>
       <c r="K4" t="n">
-        <v>0.1958372415125151</v>
+        <v>0.5333153014252645</v>
       </c>
       <c r="L4" t="n">
-        <v>0.1828094737230775</v>
+        <v>0.3690952700336221</v>
       </c>
       <c r="M4" t="n">
-        <v>0.3390171050726593</v>
+        <v>0.6151576663404461</v>
       </c>
       <c r="N4" t="n">
-        <v>0.4837186243978747</v>
+        <v>-0.6998715991523785</v>
       </c>
       <c r="O4" t="n">
-        <v>0.3534497650977566</v>
+        <v>0.6413462017484781</v>
       </c>
       <c r="P4" t="n">
-        <v>34.32681886173259</v>
+        <v>31.94350670399617</v>
       </c>
       <c r="Q4" t="n">
-        <v>52.6099562347556</v>
+        <v>50.22664407701918</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_13</t>
+          <t>model_1_3_0</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8070248139253393</v>
+        <v>0.2725587106264931</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3900816354190949</v>
+        <v>-0.1321651203373435</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7434953139655938</v>
+        <v>-2.445770544261505</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4635264523124243</v>
+        <v>-0.3184240668125458</v>
       </c>
       <c r="F5" t="n">
-        <v>0.6688356043962527</v>
+        <v>-0.1654184531408569</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1145584065479035</v>
+        <v>0.4318405731996019</v>
       </c>
       <c r="H5" t="n">
-        <v>0.3620738883167033</v>
+        <v>0.6721021224188993</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1250403738557666</v>
+        <v>0.3035867358418661</v>
       </c>
       <c r="J5" t="n">
-        <v>0.2594356047819023</v>
+        <v>0.6045012994904911</v>
       </c>
       <c r="K5" t="n">
-        <v>0.1922379893188345</v>
+        <v>0.4540440176661786</v>
       </c>
       <c r="L5" t="n">
-        <v>0.1798296041347487</v>
+        <v>0.4637481547201175</v>
       </c>
       <c r="M5" t="n">
-        <v>0.3384647788882966</v>
+        <v>0.6571457777385485</v>
       </c>
       <c r="N5" t="n">
-        <v>0.4853995038009049</v>
+        <v>-0.9398434383293517</v>
       </c>
       <c r="O5" t="n">
-        <v>0.3528739252442527</v>
+        <v>0.6851218339761707</v>
       </c>
       <c r="P5" t="n">
-        <v>34.33334097038001</v>
+        <v>31.67939760474157</v>
       </c>
       <c r="Q5" t="n">
-        <v>52.61647834340302</v>
+        <v>49.96253497776458</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_14</t>
+          <t>model_1_3_18</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.8070207559733777</v>
+        <v>0.3850284062912862</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3897883012624281</v>
+        <v>-0.1383655574599334</v>
       </c>
       <c r="D6" t="n">
-        <v>0.7442401378572904</v>
+        <v>-4.82575628797313</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4617528792734071</v>
+        <v>-0.1769111219393744</v>
       </c>
       <c r="F6" t="n">
-        <v>0.6684095816967373</v>
+        <v>-0.3512545883657123</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1145608155234823</v>
+        <v>0.3650737034151028</v>
       </c>
       <c r="H6" t="n">
-        <v>0.3622480241434765</v>
+        <v>0.6757829697398059</v>
       </c>
       <c r="I6" t="n">
-        <v>0.1246772886454561</v>
+        <v>0.5132733919910617</v>
       </c>
       <c r="J6" t="n">
-        <v>0.260293294776098</v>
+        <v>0.5396171994320225</v>
       </c>
       <c r="K6" t="n">
-        <v>0.1924852917107771</v>
+        <v>0.5264452957115421</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1807563253527686</v>
+        <v>0.3394910022708029</v>
       </c>
       <c r="M6" t="n">
-        <v>0.3384683375494409</v>
+        <v>0.6042132929811316</v>
       </c>
       <c r="N6" t="n">
-        <v>0.485388682595674</v>
+        <v>-0.6399242498899034</v>
       </c>
       <c r="O6" t="n">
-        <v>0.3528776354049694</v>
+        <v>0.6299359037572816</v>
       </c>
       <c r="P6" t="n">
-        <v>34.33329891409932</v>
+        <v>32.01531203723906</v>
       </c>
       <c r="Q6" t="n">
-        <v>52.61643628712233</v>
+        <v>50.29844941026207</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_11</t>
+          <t>model_1_3_1</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.8070482316959127</v>
+        <v>0.2869081058667567</v>
       </c>
       <c r="C7" t="n">
-        <v>0.3889899817614823</v>
+        <v>-0.1596827146936832</v>
       </c>
       <c r="D7" t="n">
-        <v>0.7438508605134047</v>
+        <v>-2.301348648417684</v>
       </c>
       <c r="E7" t="n">
-        <v>0.4667038210972456</v>
+        <v>-0.4032589561978306</v>
       </c>
       <c r="F7" t="n">
-        <v>0.6703083908095377</v>
+        <v>-0.1990080945229553</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1145445047476961</v>
+        <v>0.4233221523233827</v>
       </c>
       <c r="H7" t="n">
-        <v>0.3627219410848448</v>
+        <v>0.6884377551270042</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1248670527599664</v>
+        <v>0.290862565331924</v>
       </c>
       <c r="J7" t="n">
-        <v>0.2578990470227017</v>
+        <v>0.6433983449604811</v>
       </c>
       <c r="K7" t="n">
-        <v>0.191383049891334</v>
+        <v>0.4671304551462026</v>
       </c>
       <c r="L7" t="n">
-        <v>0.1791486735074124</v>
+        <v>0.4526851354520028</v>
       </c>
       <c r="M7" t="n">
-        <v>0.3384442417115353</v>
+        <v>0.6506321175006524</v>
       </c>
       <c r="N7" t="n">
-        <v>0.4854619511891005</v>
+        <v>-0.9015783843553153</v>
       </c>
       <c r="O7" t="n">
-        <v>0.3528525137573588</v>
+        <v>0.6783308737368117</v>
       </c>
       <c r="P7" t="n">
-        <v>34.33358368750911</v>
+        <v>31.71924360076187</v>
       </c>
       <c r="Q7" t="n">
-        <v>52.61672106053212</v>
+        <v>50.00238097378489</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_16</t>
+          <t>model_1_3_3</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.805622613644025</v>
+        <v>0.2982101484753329</v>
       </c>
       <c r="C8" t="n">
-        <v>0.3873926611636851</v>
+        <v>-0.183948659626499</v>
       </c>
       <c r="D8" t="n">
-        <v>0.7394559515359549</v>
+        <v>-2.285532380857044</v>
       </c>
       <c r="E8" t="n">
-        <v>0.4427533616583952</v>
+        <v>-0.4616682189879766</v>
       </c>
       <c r="F8" t="n">
-        <v>0.6584867376413227</v>
+        <v>-0.2315895980681808</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1153908132067899</v>
+        <v>0.4166127716081125</v>
       </c>
       <c r="H8" t="n">
-        <v>0.3636701795923543</v>
+        <v>0.7028430682733641</v>
       </c>
       <c r="I8" t="n">
-        <v>0.1270094738989262</v>
+        <v>0.2894690862884825</v>
       </c>
       <c r="J8" t="n">
-        <v>0.2694813551460113</v>
+        <v>0.6701791631719444</v>
       </c>
       <c r="K8" t="n">
-        <v>0.1982454145224688</v>
+        <v>0.4798241247302134</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1841552991852211</v>
+        <v>0.4425282059572934</v>
       </c>
       <c r="M8" t="n">
-        <v>0.3396922330680963</v>
+        <v>0.6454554760849989</v>
       </c>
       <c r="N8" t="n">
-        <v>0.4816603030507334</v>
+        <v>-0.8714396040657788</v>
       </c>
       <c r="O8" t="n">
-        <v>0.3541536346896669</v>
+        <v>0.6729338519789688</v>
       </c>
       <c r="P8" t="n">
-        <v>34.3188610726742</v>
+        <v>31.75119618772124</v>
       </c>
       <c r="Q8" t="n">
-        <v>52.60199844569721</v>
+        <v>50.03433356074425</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_17</t>
+          <t>model_1_3_2</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.8048546754512453</v>
+        <v>0.2961154071922144</v>
       </c>
       <c r="C9" t="n">
-        <v>0.3841011349065081</v>
+        <v>-0.1879503993599649</v>
       </c>
       <c r="D9" t="n">
-        <v>0.7390827471923787</v>
+        <v>-2.26456942002493</v>
       </c>
       <c r="E9" t="n">
-        <v>0.4355259396817108</v>
+        <v>-0.4638344418317226</v>
       </c>
       <c r="F9" t="n">
-        <v>0.655319531806368</v>
+        <v>-0.2304939739739986</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1158466944912265</v>
+        <v>0.4178563005218834</v>
       </c>
       <c r="H9" t="n">
-        <v>0.3656241717651453</v>
+        <v>0.705218673845305</v>
       </c>
       <c r="I9" t="n">
-        <v>0.1271914027804871</v>
+        <v>0.2876221621329549</v>
       </c>
       <c r="J9" t="n">
-        <v>0.2729764959588573</v>
+        <v>0.6711723826959146</v>
       </c>
       <c r="K9" t="n">
-        <v>0.2000839493696722</v>
+        <v>0.4793972724144347</v>
       </c>
       <c r="L9" t="n">
-        <v>0.1872699885824571</v>
+        <v>0.4440585792151993</v>
       </c>
       <c r="M9" t="n">
-        <v>0.3403625926732056</v>
+        <v>0.6464180539881939</v>
       </c>
       <c r="N9" t="n">
-        <v>0.4796124678699876</v>
+        <v>-0.8770255808207614</v>
       </c>
       <c r="O9" t="n">
-        <v>0.3548525328910014</v>
+        <v>0.6739374088163138</v>
       </c>
       <c r="P9" t="n">
-        <v>34.31097512234358</v>
+        <v>31.74523536843718</v>
       </c>
       <c r="Q9" t="n">
-        <v>52.59411249536659</v>
+        <v>50.02837274146019</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_18</t>
+          <t>model_1_3_15</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.8047076871571859</v>
+        <v>0.3854198077083959</v>
       </c>
       <c r="C10" t="n">
-        <v>0.3836941196690568</v>
+        <v>-0.1892724465105737</v>
       </c>
       <c r="D10" t="n">
-        <v>0.7391705087980907</v>
+        <v>-4.576971053045443</v>
       </c>
       <c r="E10" t="n">
-        <v>0.4342928711352255</v>
+        <v>-0.1988276221601359</v>
       </c>
       <c r="F10" t="n">
-        <v>0.6548427603394946</v>
+        <v>-0.3360206118876448</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1159339530921439</v>
+        <v>0.3648413506262457</v>
       </c>
       <c r="H10" t="n">
-        <v>0.3658657935922391</v>
+        <v>0.7060034981433696</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1271486209344395</v>
+        <v>0.4913543766569936</v>
       </c>
       <c r="J10" t="n">
-        <v>0.2735728010059074</v>
+        <v>0.5496659790297463</v>
       </c>
       <c r="K10" t="n">
-        <v>0.2003607109701735</v>
+        <v>0.5205101778433699</v>
       </c>
       <c r="L10" t="n">
-        <v>0.1878727838799379</v>
+        <v>0.3447063586276636</v>
       </c>
       <c r="M10" t="n">
-        <v>0.3404907533137191</v>
+        <v>0.6040209852531994</v>
       </c>
       <c r="N10" t="n">
-        <v>0.4792204990858291</v>
+        <v>-0.6388805127776109</v>
       </c>
       <c r="O10" t="n">
-        <v>0.3549861495953106</v>
+        <v>0.6297354090912393</v>
       </c>
       <c r="P10" t="n">
-        <v>34.30946923984735</v>
+        <v>32.01658535141674</v>
       </c>
       <c r="Q10" t="n">
-        <v>52.59260661287036</v>
+        <v>50.29972272443975</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_24</t>
+          <t>model_1_3_16</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.8024826420797458</v>
+        <v>0.3852322862947396</v>
       </c>
       <c r="C11" t="n">
-        <v>0.3828914316666234</v>
+        <v>-0.1911127787688054</v>
       </c>
       <c r="D11" t="n">
-        <v>0.7272927492897294</v>
+        <v>-4.611486735200517</v>
       </c>
       <c r="E11" t="n">
-        <v>0.4219511647608332</v>
+        <v>-0.1943677180523093</v>
       </c>
       <c r="F11" t="n">
-        <v>0.6447146761597342</v>
+        <v>-0.337298977965754</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1172548359670549</v>
+        <v>0.3649526714378953</v>
       </c>
       <c r="H11" t="n">
-        <v>0.3663423038647998</v>
+        <v>0.70709599887007</v>
       </c>
       <c r="I11" t="n">
-        <v>0.132938766574489</v>
+        <v>0.4943953520052403</v>
       </c>
       <c r="J11" t="n">
-        <v>0.2795411811265724</v>
+        <v>0.5476210999224481</v>
       </c>
       <c r="K11" t="n">
-        <v>0.2062399738505307</v>
+        <v>0.5210082259638442</v>
       </c>
       <c r="L11" t="n">
-        <v>0.1863868966446955</v>
+        <v>0.3441767684992959</v>
       </c>
       <c r="M11" t="n">
-        <v>0.3424249347916342</v>
+        <v>0.6041131280132019</v>
       </c>
       <c r="N11" t="n">
-        <v>0.473287045545989</v>
+        <v>-0.6393805698806942</v>
       </c>
       <c r="O11" t="n">
-        <v>0.3570026731830481</v>
+        <v>0.629831474559297</v>
       </c>
       <c r="P11" t="n">
-        <v>34.28681125516944</v>
+        <v>32.01597520220123</v>
       </c>
       <c r="Q11" t="n">
-        <v>52.56994862819245</v>
+        <v>50.29911257522424</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_22</t>
+          <t>model_1_3_17</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.8032460579933774</v>
+        <v>0.385045330098262</v>
       </c>
       <c r="C12" t="n">
-        <v>0.3798786907605953</v>
+        <v>-0.1912565041319747</v>
       </c>
       <c r="D12" t="n">
-        <v>0.7303326997099017</v>
+        <v>-4.644893323708849</v>
       </c>
       <c r="E12" t="n">
-        <v>0.4287447158928981</v>
+        <v>-0.1901537320214897</v>
       </c>
       <c r="F12" t="n">
-        <v>0.6488208820256351</v>
+        <v>-0.3385966439534278</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1168016393028728</v>
+        <v>0.3650636567122116</v>
       </c>
       <c r="H12" t="n">
-        <v>0.3681307970102488</v>
+        <v>0.7071813204542597</v>
       </c>
       <c r="I12" t="n">
-        <v>0.131456857830762</v>
+        <v>0.4973386115840729</v>
       </c>
       <c r="J12" t="n">
-        <v>0.2762558578256173</v>
+        <v>0.5456889749743471</v>
       </c>
       <c r="K12" t="n">
-        <v>0.2038563578281896</v>
+        <v>0.52151379327921</v>
       </c>
       <c r="L12" t="n">
-        <v>0.1865256370222722</v>
+        <v>0.3436574575557295</v>
       </c>
       <c r="M12" t="n">
-        <v>0.3417625481278966</v>
+        <v>0.6042049790528142</v>
       </c>
       <c r="N12" t="n">
-        <v>0.4753228213156733</v>
+        <v>-0.6398791197379678</v>
       </c>
       <c r="O12" t="n">
-        <v>0.3563120873477059</v>
+        <v>0.6299272358878234</v>
       </c>
       <c r="P12" t="n">
-        <v>34.29455634711833</v>
+        <v>32.01536707730926</v>
       </c>
       <c r="Q12" t="n">
-        <v>52.57769372014134</v>
+        <v>50.29850445033227</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_23</t>
+          <t>model_1_3_11</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.8031203749469744</v>
+        <v>0.3475212291628778</v>
       </c>
       <c r="C13" t="n">
-        <v>0.3791431119959503</v>
+        <v>-0.2095062989773555</v>
       </c>
       <c r="D13" t="n">
-        <v>0.7308254289536877</v>
+        <v>-2.983374791994827</v>
       </c>
       <c r="E13" t="n">
-        <v>0.4267819051030876</v>
+        <v>-0.5445361315107582</v>
       </c>
       <c r="F13" t="n">
-        <v>0.6482101838943917</v>
+        <v>-0.3592572872821151</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1168762501884426</v>
+        <v>0.3873395839842142</v>
       </c>
       <c r="H13" t="n">
-        <v>0.3685674683402902</v>
+        <v>0.7180151870245663</v>
       </c>
       <c r="I13" t="n">
-        <v>0.1312166631980432</v>
+        <v>0.3509519090731151</v>
       </c>
       <c r="J13" t="n">
-        <v>0.2772050621368492</v>
+        <v>0.708174343984438</v>
       </c>
       <c r="K13" t="n">
-        <v>0.2042108626674462</v>
+        <v>0.5295631265287766</v>
       </c>
       <c r="L13" t="n">
-        <v>0.1880958249092484</v>
+        <v>0.3855301211298637</v>
       </c>
       <c r="M13" t="n">
-        <v>0.34187168673121</v>
+        <v>0.622366117316981</v>
       </c>
       <c r="N13" t="n">
-        <v>0.4749876665252651</v>
+        <v>-0.7399433888989926</v>
       </c>
       <c r="O13" t="n">
-        <v>0.3564258722073104</v>
+        <v>0.6488615314066348</v>
       </c>
       <c r="P13" t="n">
-        <v>34.29327918926197</v>
+        <v>31.89690698543145</v>
       </c>
       <c r="Q13" t="n">
-        <v>52.57641656228498</v>
+        <v>50.18004435845446</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_21</t>
+          <t>model_1_3_4</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.8032854030494354</v>
+        <v>0.3120448406119497</v>
       </c>
       <c r="C14" t="n">
-        <v>0.3791276958653995</v>
+        <v>-0.2146680879354077</v>
       </c>
       <c r="D14" t="n">
-        <v>0.7306086665886682</v>
+        <v>-2.372307204766126</v>
       </c>
       <c r="E14" t="n">
-        <v>0.4291472688719427</v>
+        <v>-0.4971382777412048</v>
       </c>
       <c r="F14" t="n">
-        <v>0.6491044351430698</v>
+        <v>-0.2622730014115731</v>
       </c>
       <c r="G14" t="n">
-        <v>0.1167782823779789</v>
+        <v>0.4083999007282345</v>
       </c>
       <c r="H14" t="n">
-        <v>0.3685766200213273</v>
+        <v>0.7210794479277389</v>
       </c>
       <c r="I14" t="n">
-        <v>0.1313223300674441</v>
+        <v>0.2971143096733313</v>
       </c>
       <c r="J14" t="n">
-        <v>0.2760611854582184</v>
+        <v>0.686442289088</v>
       </c>
       <c r="K14" t="n">
-        <v>0.2036917577628313</v>
+        <v>0.4917782993806656</v>
       </c>
       <c r="L14" t="n">
-        <v>0.1866986427994037</v>
+        <v>0.429278182518869</v>
       </c>
       <c r="M14" t="n">
-        <v>0.3417283751431522</v>
+        <v>0.639061734676889</v>
       </c>
       <c r="N14" t="n">
-        <v>0.4754277414651611</v>
+        <v>-0.8345470917014675</v>
       </c>
       <c r="O14" t="n">
-        <v>0.356276459548253</v>
+        <v>0.6662679157622464</v>
       </c>
       <c r="P14" t="n">
-        <v>34.29495632884285</v>
+        <v>31.791016871533</v>
       </c>
       <c r="Q14" t="n">
-        <v>52.57809370186586</v>
+        <v>50.07415424455601</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_20</t>
+          <t>model_1_3_10</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.8033961733547509</v>
+        <v>0.3470213778023784</v>
       </c>
       <c r="C15" t="n">
-        <v>0.3790593799140753</v>
+        <v>-0.2181504066406093</v>
       </c>
       <c r="D15" t="n">
-        <v>0.7313543134242249</v>
+        <v>-2.967546828985461</v>
       </c>
       <c r="E15" t="n">
-        <v>0.4296450792762436</v>
+        <v>-0.54296480056285</v>
       </c>
       <c r="F15" t="n">
-        <v>0.6496248778221342</v>
+        <v>-0.3565429862866831</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1167125243397156</v>
+        <v>0.3876363173442611</v>
       </c>
       <c r="H15" t="n">
-        <v>0.3686171753211288</v>
+        <v>0.7231467027394819</v>
       </c>
       <c r="I15" t="n">
-        <v>0.1309588436901626</v>
+        <v>0.3495573996119319</v>
       </c>
       <c r="J15" t="n">
-        <v>0.2758204471331636</v>
+        <v>0.7074538841385885</v>
       </c>
       <c r="K15" t="n">
-        <v>0.2033896454116631</v>
+        <v>0.5285056418752602</v>
       </c>
       <c r="L15" t="n">
-        <v>0.186958656485129</v>
+        <v>0.3866396336690577</v>
       </c>
       <c r="M15" t="n">
-        <v>0.3416321476964889</v>
+        <v>0.6226044629973841</v>
       </c>
       <c r="N15" t="n">
-        <v>0.4757231289460024</v>
+        <v>-0.7412763258603241</v>
       </c>
       <c r="O15" t="n">
-        <v>0.3561761354999671</v>
+        <v>0.6491100239560963</v>
       </c>
       <c r="P15" t="n">
-        <v>34.29608284925582</v>
+        <v>31.8953754107126</v>
       </c>
       <c r="Q15" t="n">
-        <v>52.57922022227883</v>
+        <v>50.17851278373561</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_19</t>
+          <t>model_1_3_6</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.8034701916049917</v>
+        <v>0.3153445665669627</v>
       </c>
       <c r="C16" t="n">
-        <v>0.3786994962502106</v>
+        <v>-0.2189278088524287</v>
       </c>
       <c r="D16" t="n">
-        <v>0.7315625374189831</v>
+        <v>-2.418984654271203</v>
       </c>
       <c r="E16" t="n">
-        <v>0.4308767814699209</v>
+        <v>-0.5981974001566817</v>
       </c>
       <c r="F16" t="n">
-        <v>0.6502253597852075</v>
+        <v>-0.3270172470504766</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1166685839089508</v>
+        <v>0.4064410408605995</v>
       </c>
       <c r="H16" t="n">
-        <v>0.3688308178101637</v>
+        <v>0.7236082022744449</v>
       </c>
       <c r="I16" t="n">
-        <v>0.130857339087838</v>
+        <v>0.3012267873762559</v>
       </c>
       <c r="J16" t="n">
-        <v>0.2752248028466834</v>
+        <v>0.732778192962402</v>
       </c>
       <c r="K16" t="n">
-        <v>0.2030410709672607</v>
+        <v>0.5170024901693289</v>
       </c>
       <c r="L16" t="n">
-        <v>0.1868903434264108</v>
+        <v>0.4178947843454495</v>
       </c>
       <c r="M16" t="n">
-        <v>0.3415678320757837</v>
+        <v>0.6375272863655324</v>
       </c>
       <c r="N16" t="n">
-        <v>0.4759205109466444</v>
+        <v>-0.8257478224880992</v>
       </c>
       <c r="O16" t="n">
-        <v>0.3561090818301367</v>
+        <v>0.6646681428095295</v>
       </c>
       <c r="P16" t="n">
-        <v>34.29683595959305</v>
+        <v>31.80063280289412</v>
       </c>
       <c r="Q16" t="n">
-        <v>52.57997333261606</v>
+        <v>50.08377017591713</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_9</t>
+          <t>model_1_3_5</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.8008592832839025</v>
+        <v>0.3247660260795563</v>
       </c>
       <c r="C17" t="n">
-        <v>0.3248119567471035</v>
+        <v>-0.2353289932785729</v>
       </c>
       <c r="D17" t="n">
-        <v>0.7352886205625314</v>
+        <v>-2.518156291452902</v>
       </c>
       <c r="E17" t="n">
-        <v>0.4898021626051291</v>
+        <v>-0.4891424413439367</v>
       </c>
       <c r="F17" t="n">
-        <v>0.676334603317519</v>
+        <v>-0.2740592673972424</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1182185318737161</v>
+        <v>0.4008480555080645</v>
       </c>
       <c r="H17" t="n">
-        <v>0.4008207890797069</v>
+        <v>0.7333446538440807</v>
       </c>
       <c r="I17" t="n">
-        <v>0.1290409557831507</v>
+        <v>0.3099642216404803</v>
       </c>
       <c r="J17" t="n">
-        <v>0.2467288183611265</v>
+        <v>0.6827761746606841</v>
       </c>
       <c r="K17" t="n">
-        <v>0.1878848870721386</v>
+        <v>0.4963701981505821</v>
       </c>
       <c r="L17" t="n">
-        <v>0.1774685747406801</v>
+        <v>0.4188178594370864</v>
       </c>
       <c r="M17" t="n">
-        <v>0.3438292190517207</v>
+        <v>0.6331256237967821</v>
       </c>
       <c r="N17" t="n">
-        <v>0.4689580887570735</v>
+        <v>-0.8006239304545164</v>
       </c>
       <c r="O17" t="n">
-        <v>0.3584667407313558</v>
+        <v>0.6600790923525298</v>
       </c>
       <c r="P17" t="n">
-        <v>34.27044080451576</v>
+        <v>31.82834567485315</v>
       </c>
       <c r="Q17" t="n">
-        <v>52.55357817753877</v>
+        <v>50.11148304787616</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_8</t>
+          <t>model_1_3_7</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.8008482624620799</v>
+        <v>0.324096854223455</v>
       </c>
       <c r="C18" t="n">
-        <v>0.3246183260124256</v>
+        <v>-0.2584876623504613</v>
       </c>
       <c r="D18" t="n">
-        <v>0.7358591205193679</v>
+        <v>-2.532677341286493</v>
       </c>
       <c r="E18" t="n">
-        <v>0.4910589556633986</v>
+        <v>-0.5836746333734211</v>
       </c>
       <c r="F18" t="n">
-        <v>0.677097650506381</v>
+        <v>-0.3313269112743253</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1182250743096248</v>
+        <v>0.4012453048285651</v>
       </c>
       <c r="H18" t="n">
-        <v>0.4009357366482239</v>
+        <v>0.7470926402075673</v>
       </c>
       <c r="I18" t="n">
-        <v>0.1287628496440763</v>
+        <v>0.3112435866078658</v>
       </c>
       <c r="J18" t="n">
-        <v>0.2461210402729742</v>
+        <v>0.7261194618199232</v>
       </c>
       <c r="K18" t="n">
-        <v>0.1874419449585252</v>
+        <v>0.5186815242138945</v>
       </c>
       <c r="L18" t="n">
-        <v>0.177263060172885</v>
+        <v>0.4106009470770522</v>
       </c>
       <c r="M18" t="n">
-        <v>0.3438387329979344</v>
+        <v>0.6334392668824417</v>
       </c>
       <c r="N18" t="n">
-        <v>0.4689286998988796</v>
+        <v>-0.8024083887374531</v>
       </c>
       <c r="O18" t="n">
-        <v>0.3584766597059563</v>
+        <v>0.6604060878736766</v>
       </c>
       <c r="P18" t="n">
-        <v>34.27033012381661</v>
+        <v>31.82636461193641</v>
       </c>
       <c r="Q18" t="n">
-        <v>52.55346749683962</v>
+        <v>50.10950198495942</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_6</t>
+          <t>model_1_3_9</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.7979930758750957</v>
+        <v>0.332382415450466</v>
       </c>
       <c r="C19" t="n">
-        <v>0.306747216517995</v>
+        <v>-0.2962746102786926</v>
       </c>
       <c r="D19" t="n">
-        <v>0.7297028777560424</v>
+        <v>-2.701861118281792</v>
       </c>
       <c r="E19" t="n">
-        <v>0.5012523373287954</v>
+        <v>-0.5884996881934754</v>
       </c>
       <c r="F19" t="n">
-        <v>0.6787586835315547</v>
+        <v>-0.3532958674999773</v>
       </c>
       <c r="G19" t="n">
-        <v>0.119920036405297</v>
+        <v>0.3963266377666029</v>
       </c>
       <c r="H19" t="n">
-        <v>0.4115447992358511</v>
+        <v>0.7695246048089228</v>
       </c>
       <c r="I19" t="n">
-        <v>0.1317638821342579</v>
+        <v>0.3261493819751569</v>
       </c>
       <c r="J19" t="n">
-        <v>0.2411915779564556</v>
+        <v>0.7283317635991885</v>
       </c>
       <c r="K19" t="n">
-        <v>0.1864777300453567</v>
+        <v>0.5272405727871727</v>
       </c>
       <c r="L19" t="n">
-        <v>0.1748786484603438</v>
+        <v>0.4004586686595332</v>
       </c>
       <c r="M19" t="n">
-        <v>0.3462947247725513</v>
+        <v>0.6295447861483747</v>
       </c>
       <c r="N19" t="n">
-        <v>0.4613148690002553</v>
+        <v>-0.7803135587987573</v>
       </c>
       <c r="O19" t="n">
-        <v>0.3610372081350225</v>
+        <v>0.656345811032074</v>
       </c>
       <c r="P19" t="n">
-        <v>34.24186024321596</v>
+        <v>31.85103312975722</v>
       </c>
       <c r="Q19" t="n">
-        <v>52.52499761623897</v>
+        <v>50.13417050278023</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>model_1_3_7</t>
+          <t>model_1_3_8</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.7978393285625657</v>
+        <v>0.3270464345059314</v>
       </c>
       <c r="C20" t="n">
-        <v>0.3052950780954677</v>
+        <v>-0.3006316004122813</v>
       </c>
       <c r="D20" t="n">
-        <v>0.7299278658641829</v>
+        <v>-2.596753627988628</v>
       </c>
       <c r="E20" t="n">
-        <v>0.4986255520512417</v>
+        <v>-0.5965090740791228</v>
       </c>
       <c r="F20" t="n">
-        <v>0.6777589938817841</v>
+        <v>-0.3461242584096016</v>
       </c>
       <c r="G20" t="n">
-        <v>0.120011307451553</v>
+        <v>0.3994943065576534</v>
       </c>
       <c r="H20" t="n">
-        <v>0.4124068513325769</v>
+        <v>0.7721111023643948</v>
       </c>
       <c r="I20" t="n">
-        <v>0.1316542053966125</v>
+        <v>0.3168889743302621</v>
       </c>
       <c r="J20" t="n">
-        <v>0.2424618766134011</v>
+        <v>0.7320040905066456</v>
       </c>
       <c r="K20" t="n">
-        <v>0.1870580410050068</v>
+        <v>0.5244465324184538</v>
       </c>
       <c r="L20" t="n">
-        <v>0.1779751804204535</v>
+        <v>0.4059779513755755</v>
       </c>
       <c r="M20" t="n">
-        <v>0.3464264820298139</v>
+        <v>0.6320556198291836</v>
       </c>
       <c r="N20" t="n">
-        <v>0.4609048761668418</v>
+        <v>-0.7945428413175162</v>
       </c>
       <c r="O20" t="n">
-        <v>0.3611745745715019</v>
+        <v>0.658963536100817</v>
       </c>
       <c r="P20" t="n">
-        <v>34.24033862375281</v>
+        <v>31.835111530595</v>
       </c>
       <c r="Q20" t="n">
-        <v>52.52347599677582</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>model_1_3_5</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>0.7977347352705462</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0.3048063880263097</v>
-      </c>
-      <c r="D21" t="n">
-        <v>0.7296377942784451</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0.5023542142510732</v>
-      </c>
-      <c r="F21" t="n">
-        <v>0.6791903307521081</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0.1200733985478907</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0.4126969588679409</v>
-      </c>
-      <c r="I21" t="n">
-        <v>0.131795608893314</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0.2406587164445347</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0.1862271626689244</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0.1747610241162658</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0.3465160869972572</v>
-      </c>
-      <c r="N21" t="n">
-        <v>0.4606259607214565</v>
-      </c>
-      <c r="O21" t="n">
-        <v>0.3612679942079171</v>
-      </c>
-      <c r="P21" t="n">
-        <v>34.2393041372375</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>52.52244151026051</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>model_1_3_4</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>0.7948036195344279</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0.2913418503423056</v>
-      </c>
-      <c r="D22" t="n">
-        <v>0.7219735033668164</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0.5047231935401353</v>
-      </c>
-      <c r="F22" t="n">
-        <v>0.676958989487072</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0.1218134354664574</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0.4206900900749082</v>
-      </c>
-      <c r="I22" t="n">
-        <v>0.1355317815759482</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0.2395130913205694</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0.1875224364482588</v>
-      </c>
-      <c r="L22" t="n">
-        <v>0.173084135960291</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0.3490178153998122</v>
-      </c>
-      <c r="N22" t="n">
-        <v>0.4528096520918078</v>
-      </c>
-      <c r="O22" t="n">
-        <v>0.3638762263678606</v>
-      </c>
-      <c r="P22" t="n">
-        <v>34.21052924436679</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>52.4936666173898</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>model_1_3_3</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>0.786288112364005</v>
-      </c>
-      <c r="C23" t="n">
-        <v>0.285156858322888</v>
-      </c>
-      <c r="D23" t="n">
-        <v>0.7158853386877488</v>
-      </c>
-      <c r="E23" t="n">
-        <v>0.5107501883888304</v>
-      </c>
-      <c r="F23" t="n">
-        <v>0.6769131447256296</v>
-      </c>
-      <c r="G23" t="n">
-        <v>0.1268686083735765</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0.4243617685153781</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0.138499627502412</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0.2365984703474973</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0.1875490489249547</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0.1766627988105563</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0.3561861990217708</v>
-      </c>
-      <c r="N23" t="n">
-        <v>0.4301016329706799</v>
-      </c>
-      <c r="O23" t="n">
-        <v>0.3713497829212057</v>
-      </c>
-      <c r="P23" t="n">
-        <v>34.12920661561238</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>52.41234398863539</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>model_1_3_2</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>0.7847806284333195</v>
-      </c>
-      <c r="C24" t="n">
-        <v>0.2821355767376021</v>
-      </c>
-      <c r="D24" t="n">
-        <v>0.7161544151884536</v>
-      </c>
-      <c r="E24" t="n">
-        <v>0.5123385051374163</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0.6776877215637815</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0.1277635159547464</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0.4261553317769726</v>
-      </c>
-      <c r="I24" t="n">
-        <v>0.1383684586463413</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0.2358303692583928</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0.187099413952367</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0.1772341005532542</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0.3574402271076192</v>
-      </c>
-      <c r="N24" t="n">
-        <v>0.4260816758221855</v>
-      </c>
-      <c r="O24" t="n">
-        <v>0.3726571975788648</v>
-      </c>
-      <c r="P24" t="n">
-        <v>34.1151485109152</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>52.39828588393821</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>model_1_3_1</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>0.7426964953630729</v>
-      </c>
-      <c r="C25" t="n">
-        <v>0.0837247082741992</v>
-      </c>
-      <c r="D25" t="n">
-        <v>0.6275837171404524</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0.5461410388523382</v>
-      </c>
-      <c r="F25" t="n">
-        <v>0.6545783716470852</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0.1527464752851349</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0.5439405942000863</v>
-      </c>
-      <c r="I25" t="n">
-        <v>0.18154471935256</v>
-      </c>
-      <c r="J25" t="n">
-        <v>0.2194836531615937</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0.2005141862570768</v>
-      </c>
-      <c r="L25" t="n">
-        <v>0.1857530124790846</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0.3908279356508882</v>
-      </c>
-      <c r="N25" t="n">
-        <v>0.3138573209681945</v>
-      </c>
-      <c r="O25" t="n">
-        <v>0.4074662899969054</v>
-      </c>
-      <c r="P25" t="n">
-        <v>33.75795151250613</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>52.04108888552914</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>model_1_3_0</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>0.7262863353644655</v>
-      </c>
-      <c r="C26" t="n">
-        <v>0.02656186372466707</v>
-      </c>
-      <c r="D26" t="n">
-        <v>0.60757952052933</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0.5655742133219401</v>
-      </c>
-      <c r="F26" t="n">
-        <v>0.6542736038518026</v>
-      </c>
-      <c r="G26" t="n">
-        <v>0.1624882551423093</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0.5778749280309984</v>
-      </c>
-      <c r="I26" t="n">
-        <v>0.1912963237447054</v>
-      </c>
-      <c r="J26" t="n">
-        <v>0.2100858787641699</v>
-      </c>
-      <c r="K26" t="n">
-        <v>0.2006911012544377</v>
-      </c>
-      <c r="L26" t="n">
-        <v>0.1880020237928347</v>
-      </c>
-      <c r="M26" t="n">
-        <v>0.4030983194486294</v>
-      </c>
-      <c r="N26" t="n">
-        <v>0.2700968943052414</v>
-      </c>
-      <c r="O26" t="n">
-        <v>0.4202590494361125</v>
-      </c>
-      <c r="P26" t="n">
-        <v>33.63429911174342</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>51.91743648476643</v>
+        <v>50.11824890361801</v>
       </c>
     </row>
   </sheetData>

</xml_diff>